<commit_message>
session 22 final: SEO/legal/manifest B2B, checklist update, cursorrules B2B rewrite
</commit_message>
<xml_diff>
--- a/POTAL_B2B_Checklist.xlsx
+++ b/POTAL_B2B_Checklist.xlsx
@@ -1286,7 +1286,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="I12" s="22" t="inlineStr">
         <is>
-          <t>GPT-4o-mini + 공개 HS Code DB. 상품명/카테고리 → HS Code + 관세율</t>
+          <t>GPT-4o-mini AI 분류 + DB캐싱 + 키워드 매칭. ai-classifier-wrapper.ts</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="F13" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="I13" s="28" t="inlineStr">
         <is>
-          <t>국가코드 + HS Code(선택) → 관세율, VAT/GST, de minimis 기준</t>
+          <t>/api/v1/countries에서 세율 정보 제공. 139개국 데이터</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="I16" s="22" t="inlineStr">
         <is>
-          <t>HTS 공개 데이터 기반. Chapter 1~97</t>
+          <t>USITC REST API 연동 (usitc-provider.ts). 실시간 조회</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I18" s="28" t="inlineStr">
         <is>
-          <t>표준세율 + 경감세율. AT~SE 27국</t>
+          <t>EU TARIC API 연동 (eu-taric-provider.ts). CET 파싱</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="F19" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="I19" s="22" t="inlineStr">
         <is>
-          <t>Common External Tariff. TARIC 공개 DB</t>
+          <t>EU TARIC API에서 27개국 VAT 데이터 제공</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="I20" s="22" t="inlineStr">
         <is>
-          <t>VAT 20% 표준, UK Global Tariff</t>
+          <t>UK Trade Tariff API 연동 (uk-tariff-provider.ts). MFN 파싱</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="F33" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="I33" s="28" t="inlineStr">
         <is>
-          <t>무료 API (exchangerate-api 또는 frankfurter). 캐시 1시간</t>
+          <t>ExchangeRate-API + Fawaz CDN 이중 폴백. exchange-rate-service.ts</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="I34" s="22" t="inlineStr">
         <is>
-          <t>ISO 4217 코드 지원. 150+ 통화</t>
+          <t>166+ 통화 지원. exchange-rate-service.ts에 통합</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="I36" s="28" t="inlineStr">
         <is>
-          <t>국가별 관세율 데이터에서 HS Code로 조회</t>
+          <t>AI 분류 + 외부 API (USITC/UK/EU) 조합으로 HS→관세율 매핑</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="F37" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G37" s="29" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="I37" s="22" t="inlineStr">
         <is>
-          <t>USMCA, EU-KR, RCEP, CPTPP 등 주요 FTA 우대세율</t>
+          <t>27개 FTA 적용. fta-agreements.ts</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="F41" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="I41" s="22" t="inlineStr">
         <is>
-          <t>US, EU, UK, JP, KR, AU, CA 각 1개씩 시나리오</t>
+          <t>__tests__/api/cost-engine.test.ts 작성 완료</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G60" s="25" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="I60" s="22" t="inlineStr">
         <is>
-          <t>partners.shopify.com</t>
+          <t>Shopify Partner Dashboard 등록 완료. Client ID: 2fa34ed65342ffb7fac08dd916f470b8</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="F61" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G61" s="25" t="inlineStr">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="I61" s="22" t="inlineStr">
         <is>
-          <t>Shopify CLI + Remix 템플릿</t>
+          <t>Shopify CLI + shopify.app.toml 설정 완료</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G62" s="25" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="I62" s="28" t="inlineStr">
         <is>
-          <t>설치 → 권한 동의 → 콜백 → seller 등록</t>
+          <t>OAuth managed install flow. app/api/shopify/auth+callback. host→shop 추출</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="F63" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G63" s="25" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="I63" s="22" t="inlineStr">
         <is>
-          <t>Script Tag 또는 App Block</t>
+          <t>Theme App Extension 3블록 (상품위젯/장바구니배너/앱임베드). potal-3 릴리스</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G64" s="25" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="I64" s="28" t="inlineStr">
         <is>
-          <t>앱 리스팅, 스크린샷, 설명</t>
+          <t>앱 리스팅 전체 작성 + $19 결제 + 예비 단계 8/9. 임베디드 확인 대기</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G68" s="25" t="inlineStr">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="I68" s="22" t="inlineStr">
         <is>
-          <t>allowed_domains 체크</t>
+          <t>CORS 설정 완료. widget.js HTTP 200 + Access-Control-Allow-Origin</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4192,7 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G74" s="25" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="I74" s="22" t="inlineStr">
         <is>
-          <t>Stripe Dashboard → API Keys</t>
+          <t>Stripe 계정 가입 (Wise USD). Test mode API 키 설정 완료</t>
         </is>
       </c>
     </row>
@@ -4239,7 +4239,7 @@
       </c>
       <c r="F75" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G75" s="25" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="I75" s="22" t="inlineStr">
         <is>
-          <t>Starter/Growth/Enterprise 3개 plan</t>
+          <t>POTAL Growth $49/month product 생성 완료</t>
         </is>
       </c>
     </row>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G76" s="25" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="I76" s="22" t="inlineStr">
         <is>
-          <t>14일 무료 체험 → 자동 과금 전환</t>
+          <t>app/api/billing/checkout/route.ts 완료</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="F77" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G77" s="25" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="I77" s="22" t="inlineStr">
         <is>
-          <t>subscription.created/updated/deleted → sellers 테이블 업데이트</t>
+          <t>app/api/billing/webhook/route.ts 6개 이벤트 처리</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G78" s="25" t="inlineStr">
@@ -4393,7 +4393,11 @@
           <t>2h</t>
         </is>
       </c>
-      <c r="I78" s="22" t="n"/>
+      <c r="I78" s="22" t="inlineStr">
+        <is>
+          <t>app/lib/billing/subscription.ts 라이프사이클 관리</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="19">
       <c r="A79" s="35" t="inlineStr">
@@ -4470,7 +4474,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G80" s="25" t="inlineStr">
@@ -4485,7 +4489,7 @@
       </c>
       <c r="I80" s="28" t="inlineStr">
         <is>
-          <t>이번 달 계산 횟수, 남은 한도, 플랜 정보</t>
+          <t>Dashboard Overview/API Keys/Widget/Usage/Billing 5탭 완료</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4615,7 @@
       </c>
       <c r="F83" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G83" s="25" t="inlineStr">
@@ -4626,7 +4630,7 @@
       </c>
       <c r="I83" s="22" t="inlineStr">
         <is>
-          <t>Stripe Customer Portal 연동</t>
+          <t>Stripe Customer Portal 연동 완료</t>
         </is>
       </c>
     </row>
@@ -5379,10 +5383,10 @@
         <v>38</v>
       </c>
       <c r="C3" s="23" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D3" s="23" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E3" s="23" t="inlineStr">
         <is>
@@ -5400,10 +5404,10 @@
         <v>17</v>
       </c>
       <c r="C4" s="23" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D4" s="23" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
@@ -5421,10 +5425,10 @@
         <v>14</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D5" s="23" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E5" s="23" t="inlineStr">
         <is>
@@ -5442,10 +5446,10 @@
         <v>11</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: 세션 26 문서 업데이트 — 181개국 통합, Stripe 정지, App Bridge, PH 에셋
- session-context.md: 세션 26 전체 반영 (Stripe→Paddle, App Bridge, 181개국, PH 에셋, 작업 로그)
- .cursorrules: 세션 26 업데이트 (139→181개국, 7개 API, 443+ HS, 63 FTA, 신규 파일 매핑)
- .claude/plan.md: 137→181개국
- docs/CHANGELOG.md: 세션 22~26 엔트리 추가
- POTAL_B2B_Checklist.xlsx: 7개 태스크 완료 처리, 139→181 노트 업데이트, Summary 카운트 갱신

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/POTAL_B2B_Checklist.xlsx
+++ b/POTAL_B2B_Checklist.xlsx
@@ -1207,7 +1207,7 @@
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>calculateGlobalLandedCostAsync. 139개국 지원</t>
+          <t>calculateGlobalLandedCostAsync. 181개국 지원</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="I13" s="28" t="inlineStr">
         <is>
-          <t>/api/v1/countries에서 세율 정보 제공. 139개국 데이터</t>
+          <t>/api/v1/countries에서 세율 정보 제공. 181개국 데이터</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="F21" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G21" s="29" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="I21" s="28" t="inlineStr">
         <is>
-          <t>소비세 10% (식품 8%), Japan Customs Tariff Schedule</t>
+          <t>Japan Customs Provider (japan-customs-provider.ts) 추가 완료. 세션 25</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G22" s="29" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="I22" s="28" t="inlineStr">
         <is>
-          <t>부가세 10%, 관세법 별표. 관세청 공개 데이터</t>
+          <t>Korea KCS Provider (korea-kcs-provider.ts) 추가 완료. 세션 25</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="F23" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G23" s="29" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="I23" s="22" t="inlineStr">
         <is>
-          <t>GST 10%, Australian Customs Tariff</t>
+          <t>Australia ABF Provider (australia-abf-provider.ts) 추가 완료. GST 10%. 세션 25</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="I24" s="28" t="inlineStr">
         <is>
-          <t>연방 GST 5% + 주별 PST/HST 가변</t>
+          <t>Canada CBSA Provider (canada-cbsa-provider.ts) 추가 완료. GST 5% + 주별 PST/HST. 세션 25</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G26" s="29" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="I26" s="22" t="inlineStr">
         <is>
-          <t>GST 5~28%, Basic Customs Duty</t>
+          <t>India 세금 구현 완료: BCD + SWS(10%) + IGST(5-28%) 캐스케이딩. 세션 25</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="I32" s="22" t="inlineStr">
         <is>
-          <t>country-data.ts에 139개국 deMinimisUsd 포함</t>
+          <t>country-data.ts에 181개국 deMinimisUsd 포함</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="I35" s="28" t="inlineStr">
         <is>
-          <t>GlobalCostEngine.ts. 139개국 DB-backed + fallback hardcoded data</t>
+          <t>GlobalCostEngine.ts. 181개국 DB-backed + fallback hardcoded data. India/Brazil 특수 세금</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="I37" s="22" t="inlineStr">
         <is>
-          <t>27개 FTA 적용. fta-agreements.ts</t>
+          <t>63개 FTA 적용. fta-agreements.ts. 세션 25에서 확장</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G40" s="31" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="I40" s="22" t="inlineStr">
         <is>
-          <t>swagger-ui-react 사용. 셀러가 바로 테스트</t>
+          <t>/developers/docs Swagger UI 스타일 재구축 완료. 6개 엔드포인트, Try it, cURL/JS/Python. 세션 24</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="I48" s="22" t="inlineStr">
         <is>
-          <t>Gemini Gem 생성 완료. 지침 + country-duty-reference.csv 업로드</t>
+          <t>Gemini Gem 생성 완료. 지침 + country-duty-reference.csv (181개국) 업로드. 세션 26 업데이트</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="I64" s="28" t="inlineStr">
         <is>
-          <t>앱 리스팅 전체 작성 + $19 결제 + 예비 단계 8/9. 임베디드 확인 대기</t>
+          <t>앱 리스팅 전체 작성 + $19 결제 + 예비 단계 8/9. App Bridge push 완료, 임베디드 확인 대기</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="I66" s="22" t="inlineStr">
         <is>
-          <t>iframe/Shadow DOM. 139개국 hardcoded. breakdown 표시</t>
+          <t>iframe/Shadow DOM. 181개국 hardcoded. breakdown 표시</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="I74" s="22" t="inlineStr">
         <is>
-          <t>Stripe 계정 가입 (Wise USD). Test mode API 키 설정 완료</t>
+          <t>⚠️ Stripe 계정 정지됨 (세션 26). Paddle/LemonSqueezy 전환 필요</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,11 @@
           <t>4h</t>
         </is>
       </c>
-      <c r="I89" s="22" t="n"/>
+      <c r="I89" s="22" t="inlineStr">
+        <is>
+          <t>country-data.ts에 181개국 포함. TH/VN/PH/ID/MY/SG 모두 세율 데이터 있음</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="19">
       <c r="A90" s="36" t="inlineStr">
@@ -4992,7 +4996,11 @@
           <t>4h</t>
         </is>
       </c>
-      <c r="I91" s="22" t="n"/>
+      <c r="I91" s="22" t="inlineStr">
+        <is>
+          <t>country-data.ts에 181개국 포함. BR/MX/AR/CL/CO 모두 세율 데이터 있음. Brazil ICMS/IPI 구현됨</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="19">
       <c r="A92" s="36" t="inlineStr">
@@ -5035,7 +5043,11 @@
           <t>3h</t>
         </is>
       </c>
-      <c r="I92" s="22" t="n"/>
+      <c r="I92" s="22" t="inlineStr">
+        <is>
+          <t>country-data.ts에 181개국 포함. ZA/NG/KE/EG 모두 세율 데이터 있음</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="19">
       <c r="A93" s="36" t="inlineStr">
@@ -5155,7 +5167,7 @@
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G95" s="31" t="inlineStr">
@@ -5168,7 +5180,11 @@
           <t>4h</t>
         </is>
       </c>
-      <c r="I95" s="22" t="n"/>
+      <c r="I95" s="22" t="inlineStr">
+        <is>
+          <t>63개 FTA 확장 완료 (27→63). 세션 25</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="19">
       <c r="A96" s="36" t="inlineStr">
@@ -5383,10 +5399,10 @@
         <v>38</v>
       </c>
       <c r="C3" s="23" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D3" s="23" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E3" s="23" t="inlineStr">
         <is>
@@ -5407,7 +5423,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
@@ -5467,10 +5483,10 @@
         <v>14</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: Stripe→LemonSqueezy 문서 전체 업데이트 (12개 파일)
- .cursorrules: 기술스택/빌링파일매핑/프로덕션환경 LS 반영
- POTAL_B2B_Checklist.xlsx: Phase 4 태스크 6개 LS 전환, Summary 갱신
- MORNING-TODO.md: ITIN→LS 전환 완료 + 후속 TODO
- app/privacy/page.tsx: Stripe→LemonSqueezy (MoR) 4곳
- app/partners/page.tsx: 기술파트너 LS 변경
- app/lib/api-auth/plan-checker.ts: 주석 수정
- i18n 5개 언어: hero.title/footer.tagline/pricing FAQ 업데이트
- PRODUCT_HUNT_LAUNCH_PLAN.md: tagline 업데이트

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/POTAL_B2B_Checklist.xlsx
+++ b/POTAL_B2B_Checklist.xlsx
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B74" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="D74" s="22" t="inlineStr">
         <is>
-          <t>Stripe 계정 연동 + API 키 설정</t>
+          <t>LemonSqueezy 계정 설정 + Store 생성</t>
         </is>
       </c>
       <c r="E74" s="22" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="I74" s="22" t="inlineStr">
         <is>
-          <t>⚠️ Stripe 계정 정지됨 (세션 26). Paddle/LemonSqueezy 전환 필요</t>
+          <t>✅ Stripe→LemonSqueezy 전환 완료 (세션 26). potalapp.lemonsqueezy.com Store #308025. 신원 확인 대기</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="B75" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
@@ -4229,17 +4229,17 @@
       </c>
       <c r="D75" s="22" t="inlineStr">
         <is>
-          <t>Stripe Products + Prices 생성</t>
+          <t>LemonSqueezy Products + Variants 생성</t>
         </is>
       </c>
       <c r="E75" s="22" t="inlineStr">
         <is>
-          <t>app/lib/billing/stripe-setup.ts</t>
+          <t>LemonSqueezy Dashboard</t>
         </is>
       </c>
       <c r="F75" s="30" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="G75" s="25" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="I75" s="22" t="inlineStr">
         <is>
-          <t>POTAL Growth $49/month product 생성 완료</t>
+          <t>Starter $9, Growth $29, Enterprise custom. 신원 확인 승인 후 생성 가능</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B76" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="D76" s="22" t="inlineStr">
         <is>
-          <t>Stripe Checkout 세션 생성</t>
+          <t>LemonSqueezy Checkout 구현</t>
         </is>
       </c>
       <c r="E76" s="22" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="I76" s="22" t="inlineStr">
         <is>
-          <t>app/api/billing/checkout/route.ts 완료</t>
+          <t>✅ app/api/billing/checkout/route.ts LemonSqueezy createCheckout() 전환 완료</t>
         </is>
       </c>
     </row>
@@ -4313,7 +4313,7 @@
       </c>
       <c r="B77" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="D77" s="22" t="inlineStr">
         <is>
-          <t>Stripe Webhook 처리</t>
+          <t>LemonSqueezy Webhook 처리</t>
         </is>
       </c>
       <c r="E77" s="22" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="I77" s="22" t="inlineStr">
         <is>
-          <t>app/api/billing/webhook/route.ts 6개 이벤트 처리</t>
+          <t>✅ app/api/billing/webhook/route.ts HMAC SHA-256 검증 + 6개 이벤트 처리</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="B78" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C78" s="23" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="D78" s="28" t="inlineStr">
         <is>
-          <t>구독 상태 관리 (trialing→active→past_due→canceled)</t>
+          <t>구독 상태 관리 (on_trial→active→past_due→cancelled)</t>
         </is>
       </c>
       <c r="E78" s="22" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="I78" s="22" t="inlineStr">
         <is>
-          <t>app/lib/billing/subscription.ts 라이프사이클 관리</t>
+          <t>✅ app/lib/billing/subscription.ts LemonSqueezy 상태 매핑 + DB billing_* 컬럼</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="B79" s="22" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>LemonSqueezy</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="D79" s="28" t="inlineStr">
         <is>
-          <t>인보이스 자동 발행</t>
+          <t>인보이스 자동 발행 (LemonSqueezy MoR 처리)</t>
         </is>
       </c>
       <c r="E79" s="22" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="F79" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G79" s="29" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="I79" s="22" t="inlineStr">
         <is>
-          <t>Stripe 자동 처리, 이메일 설정만</t>
+          <t>LemonSqueezy가 MoR로 인보이스/세금 자동 처리. 별도 설정 불필요</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="I83" s="22" t="inlineStr">
         <is>
-          <t>Stripe Customer Portal 연동 완료</t>
+          <t>✅ LemonSqueezy Customer Portal 연동 완료. subscription.urls.customer_portal</t>
         </is>
       </c>
     </row>
@@ -5462,10 +5462,10 @@
         <v>11</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>

</xml_diff>